<commit_message>
Added new RDF data schemes and visual schemes for economy-table131-133, fixed XLSX spreadsheets for economy-table131-133
</commit_message>
<xml_diff>
--- a/sources/table_normalization/xlsx/economy-table131.xlsx
+++ b/sources/table_normalization/xlsx/economy-table131.xlsx
@@ -5959,9 +5959,9 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <numFmts count="3">
-    <numFmt numFmtId="168" formatCode="#0.000"/>
-    <numFmt numFmtId="169" formatCode="#0.0"/>
-    <numFmt numFmtId="170" formatCode="#0.00"/>
+    <numFmt numFmtId="164" formatCode="#0.000"/>
+    <numFmt numFmtId="165" formatCode="#0.0"/>
+    <numFmt numFmtId="166" formatCode="#0.00"/>
   </numFmts>
   <fonts count="3">
     <font>
@@ -6015,7 +6015,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="27">
+  <cellXfs count="28">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -6035,7 +6035,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
-    <xf numFmtId="168" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
@@ -6062,20 +6062,29 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left" wrapText="1" indent="8"/>
     </xf>
-    <xf numFmtId="169" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="170" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
@@ -6083,17 +6092,11 @@
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -6378,101 +6381,101 @@
       <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="21" t="s">
+      <c r="B1" s="24" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="21"/>
-      <c r="D1" s="21"/>
-      <c r="E1" s="21"/>
-      <c r="F1" s="21"/>
-      <c r="G1" s="21"/>
-      <c r="H1" s="21"/>
-      <c r="I1" s="21"/>
-      <c r="J1" s="21"/>
-      <c r="K1" s="21"/>
-      <c r="L1" s="21"/>
-      <c r="M1" s="21"/>
-      <c r="N1" s="21"/>
-      <c r="O1" s="21"/>
-      <c r="P1" s="21"/>
-      <c r="Q1" s="21"/>
-      <c r="R1" s="21"/>
-      <c r="S1" s="21"/>
-      <c r="T1" s="21"/>
-      <c r="U1" s="21"/>
-      <c r="V1" s="21"/>
-      <c r="W1" s="21"/>
-      <c r="X1" s="21"/>
-      <c r="Y1" s="21"/>
-      <c r="Z1" s="21"/>
-      <c r="AA1" s="21"/>
-      <c r="AB1" s="21"/>
-      <c r="AC1" s="21"/>
-      <c r="AD1" s="21"/>
-      <c r="AE1" s="21"/>
-      <c r="AF1" s="21"/>
-      <c r="AG1" s="21"/>
-      <c r="AH1" s="21"/>
-      <c r="AI1" s="21"/>
-      <c r="AJ1" s="21"/>
-      <c r="AK1" s="21"/>
-      <c r="AL1" s="21"/>
-      <c r="AM1" s="21"/>
-      <c r="AN1" s="21"/>
-      <c r="AO1" s="21"/>
-      <c r="AP1" s="21"/>
-      <c r="AQ1" s="21"/>
-      <c r="AR1" s="21"/>
+      <c r="C1" s="24"/>
+      <c r="D1" s="24"/>
+      <c r="E1" s="24"/>
+      <c r="F1" s="24"/>
+      <c r="G1" s="24"/>
+      <c r="H1" s="24"/>
+      <c r="I1" s="24"/>
+      <c r="J1" s="24"/>
+      <c r="K1" s="24"/>
+      <c r="L1" s="24"/>
+      <c r="M1" s="24"/>
+      <c r="N1" s="24"/>
+      <c r="O1" s="24"/>
+      <c r="P1" s="24"/>
+      <c r="Q1" s="24"/>
+      <c r="R1" s="24"/>
+      <c r="S1" s="24"/>
+      <c r="T1" s="24"/>
+      <c r="U1" s="24"/>
+      <c r="V1" s="24"/>
+      <c r="W1" s="24"/>
+      <c r="X1" s="24"/>
+      <c r="Y1" s="24"/>
+      <c r="Z1" s="24"/>
+      <c r="AA1" s="24"/>
+      <c r="AB1" s="24"/>
+      <c r="AC1" s="24"/>
+      <c r="AD1" s="24"/>
+      <c r="AE1" s="24"/>
+      <c r="AF1" s="24"/>
+      <c r="AG1" s="24"/>
+      <c r="AH1" s="24"/>
+      <c r="AI1" s="24"/>
+      <c r="AJ1" s="24"/>
+      <c r="AK1" s="24"/>
+      <c r="AL1" s="24"/>
+      <c r="AM1" s="24"/>
+      <c r="AN1" s="24"/>
+      <c r="AO1" s="24"/>
+      <c r="AP1" s="24"/>
+      <c r="AQ1" s="24"/>
+      <c r="AR1" s="24"/>
     </row>
     <row r="2" spans="1:44" ht="15.75" customHeight="1">
       <c r="A2" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="B2" s="21" t="s">
+      <c r="B2" s="24" t="s">
         <v>2</v>
       </c>
-      <c r="C2" s="21"/>
-      <c r="D2" s="21"/>
-      <c r="E2" s="21"/>
-      <c r="F2" s="21"/>
-      <c r="G2" s="21"/>
-      <c r="H2" s="21"/>
-      <c r="I2" s="21"/>
-      <c r="J2" s="21"/>
-      <c r="K2" s="21"/>
-      <c r="L2" s="21"/>
-      <c r="M2" s="21"/>
-      <c r="N2" s="21"/>
-      <c r="O2" s="21"/>
-      <c r="P2" s="21"/>
-      <c r="Q2" s="21"/>
-      <c r="R2" s="21"/>
-      <c r="S2" s="21"/>
-      <c r="T2" s="21"/>
-      <c r="U2" s="21"/>
-      <c r="V2" s="21"/>
-      <c r="W2" s="21"/>
-      <c r="X2" s="21"/>
-      <c r="Y2" s="21"/>
-      <c r="Z2" s="21"/>
-      <c r="AA2" s="21"/>
-      <c r="AB2" s="21"/>
-      <c r="AC2" s="21"/>
-      <c r="AD2" s="21"/>
-      <c r="AE2" s="21"/>
-      <c r="AF2" s="21"/>
-      <c r="AG2" s="21"/>
-      <c r="AH2" s="21"/>
-      <c r="AI2" s="21"/>
-      <c r="AJ2" s="21"/>
-      <c r="AK2" s="21"/>
-      <c r="AL2" s="21"/>
-      <c r="AM2" s="21"/>
-      <c r="AN2" s="21"/>
-      <c r="AO2" s="21"/>
-      <c r="AP2" s="21"/>
-      <c r="AQ2" s="21"/>
-      <c r="AR2" s="21"/>
+      <c r="C2" s="24"/>
+      <c r="D2" s="24"/>
+      <c r="E2" s="24"/>
+      <c r="F2" s="24"/>
+      <c r="G2" s="24"/>
+      <c r="H2" s="24"/>
+      <c r="I2" s="24"/>
+      <c r="J2" s="24"/>
+      <c r="K2" s="24"/>
+      <c r="L2" s="24"/>
+      <c r="M2" s="24"/>
+      <c r="N2" s="24"/>
+      <c r="O2" s="24"/>
+      <c r="P2" s="24"/>
+      <c r="Q2" s="24"/>
+      <c r="R2" s="24"/>
+      <c r="S2" s="24"/>
+      <c r="T2" s="24"/>
+      <c r="U2" s="24"/>
+      <c r="V2" s="24"/>
+      <c r="W2" s="24"/>
+      <c r="X2" s="24"/>
+      <c r="Y2" s="24"/>
+      <c r="Z2" s="24"/>
+      <c r="AA2" s="24"/>
+      <c r="AB2" s="24"/>
+      <c r="AC2" s="24"/>
+      <c r="AD2" s="24"/>
+      <c r="AE2" s="24"/>
+      <c r="AF2" s="24"/>
+      <c r="AG2" s="24"/>
+      <c r="AH2" s="24"/>
+      <c r="AI2" s="24"/>
+      <c r="AJ2" s="24"/>
+      <c r="AK2" s="24"/>
+      <c r="AL2" s="24"/>
+      <c r="AM2" s="24"/>
+      <c r="AN2" s="24"/>
+      <c r="AO2" s="24"/>
+      <c r="AP2" s="24"/>
+      <c r="AQ2" s="24"/>
+      <c r="AR2" s="24"/>
     </row>
     <row r="3" spans="1:44">
       <c r="A3" s="2" t="s">
@@ -6483,74 +6486,74 @@
       </c>
     </row>
     <row r="4" spans="1:44" s="1" customFormat="1" ht="63" customHeight="1">
-      <c r="A4" s="22" t="s">
+      <c r="A4" s="19" t="s">
         <v>3</v>
       </c>
-      <c r="B4" s="22" t="s">
+      <c r="B4" s="19" t="s">
         <v>4</v>
       </c>
-      <c r="C4" s="22" t="s">
+      <c r="C4" s="19" t="s">
         <v>5</v>
       </c>
-      <c r="D4" s="23" t="s">
+      <c r="D4" s="25" t="s">
         <v>6</v>
       </c>
-      <c r="E4" s="23"/>
-      <c r="F4" s="23"/>
-      <c r="G4" s="23"/>
-      <c r="H4" s="23"/>
-      <c r="I4" s="23"/>
-      <c r="J4" s="23"/>
-      <c r="K4" s="23"/>
-      <c r="L4" s="23"/>
-      <c r="M4" s="23"/>
-      <c r="N4" s="23"/>
-      <c r="O4" s="23"/>
-      <c r="P4" s="23"/>
-      <c r="Q4" s="23" t="s">
+      <c r="E4" s="25"/>
+      <c r="F4" s="25"/>
+      <c r="G4" s="25"/>
+      <c r="H4" s="25"/>
+      <c r="I4" s="25"/>
+      <c r="J4" s="25"/>
+      <c r="K4" s="25"/>
+      <c r="L4" s="25"/>
+      <c r="M4" s="25"/>
+      <c r="N4" s="25"/>
+      <c r="O4" s="25"/>
+      <c r="P4" s="25"/>
+      <c r="Q4" s="25" t="s">
         <v>7</v>
       </c>
-      <c r="R4" s="23"/>
-      <c r="S4" s="23"/>
-      <c r="T4" s="23"/>
-      <c r="U4" s="23"/>
-      <c r="V4" s="23"/>
-      <c r="W4" s="23"/>
-      <c r="X4" s="23"/>
-      <c r="Y4" s="23"/>
-      <c r="Z4" s="23"/>
-      <c r="AA4" s="23"/>
-      <c r="AB4" s="23"/>
-      <c r="AC4" s="23"/>
-      <c r="AD4" s="22" t="s">
+      <c r="R4" s="25"/>
+      <c r="S4" s="25"/>
+      <c r="T4" s="25"/>
+      <c r="U4" s="25"/>
+      <c r="V4" s="25"/>
+      <c r="W4" s="25"/>
+      <c r="X4" s="25"/>
+      <c r="Y4" s="25"/>
+      <c r="Z4" s="25"/>
+      <c r="AA4" s="25"/>
+      <c r="AB4" s="25"/>
+      <c r="AC4" s="25"/>
+      <c r="AD4" s="21" t="s">
         <v>8</v>
       </c>
-      <c r="AE4" s="22" t="s">
+      <c r="AE4" s="21" t="s">
         <v>8</v>
       </c>
-      <c r="AF4" s="22" t="s">
+      <c r="AF4" s="21" t="s">
         <v>8</v>
       </c>
-      <c r="AG4" s="22" t="s">
+      <c r="AG4" s="21" t="s">
         <v>8</v>
       </c>
-      <c r="AH4" s="23" t="s">
+      <c r="AH4" s="25" t="s">
         <v>9</v>
       </c>
-      <c r="AI4" s="23"/>
-      <c r="AJ4" s="23"/>
-      <c r="AK4" s="19" t="s">
+      <c r="AI4" s="25"/>
+      <c r="AJ4" s="25"/>
+      <c r="AK4" s="26" t="s">
         <v>10</v>
       </c>
-      <c r="AL4" s="19"/>
-      <c r="AM4" s="19"/>
-      <c r="AN4" s="19"/>
-      <c r="AO4" s="20" t="s">
+      <c r="AL4" s="26"/>
+      <c r="AM4" s="26"/>
+      <c r="AN4" s="26"/>
+      <c r="AO4" s="27" t="s">
         <v>11</v>
       </c>
-      <c r="AP4" s="20"/>
-      <c r="AQ4" s="20"/>
-      <c r="AR4" s="20"/>
+      <c r="AP4" s="27"/>
+      <c r="AQ4" s="27"/>
+      <c r="AR4" s="27"/>
     </row>
     <row r="5" spans="1:44" s="1" customFormat="1" ht="78.75" customHeight="1">
       <c r="D5" s="4" t="s">
@@ -6652,42 +6655,42 @@
       <c r="AJ5" s="4" t="s">
         <v>28</v>
       </c>
-      <c r="AK5" s="22" t="s">
+      <c r="AK5" s="19" t="s">
         <v>29</v>
       </c>
-      <c r="AL5" s="22" t="s">
+      <c r="AL5" s="19" t="s">
         <v>30</v>
       </c>
-      <c r="AM5" s="22" t="s">
+      <c r="AM5" s="19" t="s">
         <v>31</v>
       </c>
-      <c r="AN5" s="22" t="s">
+      <c r="AN5" s="19" t="s">
         <v>31</v>
       </c>
-      <c r="AO5" s="22" t="s">
+      <c r="AO5" s="19" t="s">
         <v>32</v>
       </c>
-      <c r="AP5" s="22" t="s">
+      <c r="AP5" s="19" t="s">
         <v>30</v>
       </c>
-      <c r="AQ5" s="22" t="s">
+      <c r="AQ5" s="19" t="s">
         <v>33</v>
       </c>
-      <c r="AR5" s="22" t="s">
+      <c r="AR5" s="19" t="s">
         <v>33</v>
       </c>
     </row>
     <row r="6" spans="1:44">
-      <c r="AM6" s="22" t="s">
+      <c r="AM6" s="19" t="s">
         <v>34</v>
       </c>
-      <c r="AN6" s="22" t="s">
+      <c r="AN6" s="19" t="s">
         <v>35</v>
       </c>
-      <c r="AQ6" s="22" t="s">
+      <c r="AQ6" s="19" t="s">
         <v>34</v>
       </c>
-      <c r="AR6" s="22" t="s">
+      <c r="AR6" s="19" t="s">
         <v>35</v>
       </c>
     </row>
@@ -51282,10 +51285,10 @@
       </c>
     </row>
     <row r="349" spans="1:44">
-      <c r="A349" s="25">
+      <c r="A349" s="22">
         <v>0</v>
       </c>
-      <c r="B349" s="26" t="s">
+      <c r="B349" s="23" t="s">
         <v>467</v>
       </c>
     </row>
@@ -57197,7 +57200,7 @@
       <c r="A396" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="B396" s="24" t="s">
+      <c r="B396" s="20" t="s">
         <v>516</v>
       </c>
     </row>
@@ -57205,7 +57208,7 @@
       <c r="A397" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="B397" s="24" t="s">
+      <c r="B397" s="20" t="s">
         <v>517</v>
       </c>
     </row>
@@ -57213,7 +57216,7 @@
       <c r="A398" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="B398" s="24" t="s">
+      <c r="B398" s="20" t="s">
         <v>518</v>
       </c>
     </row>
@@ -57221,7 +57224,7 @@
       <c r="A399" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="B399" s="24" t="s">
+      <c r="B399" s="20" t="s">
         <v>519</v>
       </c>
     </row>
@@ -57229,7 +57232,7 @@
       <c r="A400" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="B400" s="24" t="s">
+      <c r="B400" s="20" t="s">
         <v>520</v>
       </c>
     </row>
@@ -57237,7 +57240,7 @@
       <c r="A401" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="B401" s="24" t="s">
+      <c r="B401" s="20" t="s">
         <v>521</v>
       </c>
     </row>
@@ -57245,7 +57248,7 @@
       <c r="A402" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="B402" s="24" t="s">
+      <c r="B402" s="20" t="s">
         <v>522</v>
       </c>
     </row>
@@ -57253,7 +57256,7 @@
       <c r="A403" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="B403" s="24" t="s">
+      <c r="B403" s="20" t="s">
         <v>523</v>
       </c>
     </row>
@@ -57261,7 +57264,7 @@
       <c r="A404" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="B404" s="24" t="s">
+      <c r="B404" s="20" t="s">
         <v>524</v>
       </c>
     </row>
@@ -57269,7 +57272,7 @@
       <c r="A405" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="B405" s="24" t="s">
+      <c r="B405" s="20" t="s">
         <v>525</v>
       </c>
     </row>
@@ -57277,7 +57280,7 @@
       <c r="A406" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="B406" s="24" t="s">
+      <c r="B406" s="20" t="s">
         <v>526</v>
       </c>
     </row>
@@ -57285,7 +57288,7 @@
       <c r="A407" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="B407" s="24" t="s">
+      <c r="B407" s="20" t="s">
         <v>527</v>
       </c>
     </row>
@@ -57293,7 +57296,7 @@
       <c r="A408" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="B408" s="24" t="s">
+      <c r="B408" s="20" t="s">
         <v>528</v>
       </c>
     </row>
@@ -57301,7 +57304,7 @@
       <c r="A409" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="B409" s="24" t="s">
+      <c r="B409" s="20" t="s">
         <v>529</v>
       </c>
     </row>
@@ -57309,7 +57312,7 @@
       <c r="A410" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="B410" s="24" t="s">
+      <c r="B410" s="20" t="s">
         <v>530</v>
       </c>
     </row>
@@ -57317,7 +57320,7 @@
       <c r="A411" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="B411" s="24" t="s">
+      <c r="B411" s="20" t="s">
         <v>531</v>
       </c>
     </row>
@@ -57325,7 +57328,7 @@
       <c r="A412" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="B412" s="24" t="s">
+      <c r="B412" s="20" t="s">
         <v>532</v>
       </c>
     </row>
@@ -57333,7 +57336,7 @@
       <c r="A413" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="B413" s="24" t="s">
+      <c r="B413" s="20" t="s">
         <v>533</v>
       </c>
     </row>
@@ -57341,7 +57344,7 @@
       <c r="A414" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="B414" s="24" t="s">
+      <c r="B414" s="20" t="s">
         <v>534</v>
       </c>
     </row>

</xml_diff>